<commit_message>
Actualización automática: 2026-04-13 14:37:35
</commit_message>
<xml_diff>
--- a/Trendmicro/Salidas_Playbooks/reporte_trendmicro.xlsx
+++ b/Trendmicro/Salidas_Playbooks/reporte_trendmicro.xlsx
@@ -429,9 +429,9 @@
   <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
@@ -520,62 +520,62 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>mongodb_qa_micro01</t>
+          <t>GEODB-CENTRAL-QA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>mongodb_qa_micro01</t>
+          <t>geodbqa</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>10.181.34.51</t>
+          <t>10.181.11.114</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>No instalado</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>No instalado</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>20.0.3</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>860.ol8</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>20.0.3</t>
-        </is>
-      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>860.ol8</t>
+          <t>5660.ol9</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1.2.0.1253</t>
+          <t>No instalado</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1.2.0.1253</t>
+          <t>1.2.0.956</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t>no activo</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>active</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>no activo</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática: 2026-04-14 15:14:20
</commit_message>
<xml_diff>
--- a/Trendmicro/Salidas_Playbooks/reporte_trendmicro.xlsx
+++ b/Trendmicro/Salidas_Playbooks/reporte_trendmicro.xlsx
@@ -431,7 +431,7 @@
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
@@ -520,7 +520,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GEODB-CENTRAL-QA</t>
+          <t>TESTGEODBCENTRAL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -530,7 +530,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>10.181.11.114</t>
+          <t>10.181.11.97</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -545,12 +545,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>20.0.3</t>
+          <t>No instalado</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>5660.ol9</t>
+          <t>No instalado</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -580,7 +580,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>desconocido</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">

</xml_diff>